<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@c69f96c3b58f776a2864e15a16ffe2a766f8e6b8 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-MedicationRequest.xlsx
+++ b/StructureDefinition-MedicationRequest.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-24T09:20:45+00:00</t>
+    <t>2024-11-25T09:16:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -8780,7 +8780,7 @@
         <v>95</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>85</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@3f17b5ad31e6abf794b31b8548163d737ac173ee 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-MedicationRequest.xlsx
+++ b/StructureDefinition-MedicationRequest.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5350" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5350" uniqueCount="804">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-12-23T15:35:28+00:00</t>
+    <t>2024-12-27T09:44:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1756,25 +1756,17 @@
     <t>MedicationRequest.dosageInstruction</t>
   </si>
   <si>
-    <t xml:space="preserve">Gebruiksinstructie
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dosage {http://nictiz.nl/fhir/StructureDefinition/zib-InstructionsForUse}
 </t>
   </si>
   <si>
-    <t>InstructionsForUse</t>
+    <t>How the medication should be taken</t>
   </si>
   <si>
     <t>Instructions for the use of the medication, e.g. dose and route of administration</t>
   </si>
   <si>
-    <t>The wiki page https://informatiestandaarden.nictiz.nl/wiki/mp:V9.0_Voorbeelden_doseringen provides dosage instruction examples. These examples consists of functional data and their representation in FHIR and CDA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() | (children().count() &gt; id.count())}
-</t>
+    <t>There are examples where a medication request may include the option of an oral dose or an Intravenous or Intramuscular dose.  For example, "Ondansetron 8mg orally or IV twice a day as needed for nausea" or "Compazine® (prochlorperazine) 5-10mg PO or 25mg PR bid prn nausea or vomiting".  In these cases, two medication requests would be created that could be grouped together.  The decision on which dose and route of administration to use is based on the patient's condition at the time the dose is needed.</t>
   </si>
   <si>
     <t>NL-CM:9.6.23240</t>
@@ -1783,7 +1775,10 @@
     <t>NL-CM:0.0.14</t>
   </si>
   <si>
-    <t>.outboundRelationship[typeCode=COMP].target[classCode=SBADM, moodCode=INT]</t>
+    <t>…occurrence[x]</t>
+  </si>
+  <si>
+    <t>see dosageInstruction mapping</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.id</t>
@@ -1871,21 +1866,17 @@
     <t>MedicationRequest.dosageInstruction.timing</t>
   </si>
   <si>
-    <t xml:space="preserve">Toedieningsschema
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Timing {http://nictiz.nl/fhir/StructureDefinition/zib-AdministrationSchedule}
 </t>
   </si>
   <si>
-    <t>AdministeringSchedule</t>
+    <t>When medication should be administered</t>
   </si>
   <si>
     <t>Specifications of the times at which the medication is to be administered. This is indicated as follows:                  Time(s) (16:00) or indications (“before meals”) at which the medication is to be taken each day.                 A specific number of times the medication is to be taken each day (“3x a day“), indicated with the frequency                 A time interval between consecutive doses (“Every 2 hours”, “every 3 days”), indicated with the word Interval.                 Combined periods with an interval and duration (“1 daily for three out of four weeks: the pill schedule”)                                                   If a certain medication is not to be taken daily, the aforementioned can be combined with daily indications:                  One or more week days on which the medication is to be administered (e.g. “Monday, Wednesday, Friday”)                 ”3x a week”, “2x a month”.                                                   The specified administration “infinite” is automatically to be repeated until:                  The end date and time has been reached                 The total administration duration has been reached (14 days)                                                   A specific amount of administrations has been reached (“20 doses”, “one-time only”), to be entered in the NumberOfDoses concept.</t>
   </si>
   <si>
-    <t>A timing schedule can be either a list of events - intervals on which the event occurs, or a single event with repeating criteria or just repeating criteria with no actual event.  When both event and a repeating specification are provided, the list of events should be understood as an interpretation of the information in the repeat structure.</t>
+    <t>This attribute may not always be populated while the Dosage.text is expected to be populated.  If both are populated, then the Dosage.text should reflect the content of the Dosage.timing.</t>
   </si>
   <si>
     <t>The timing schedule for giving the medication to the patient. The Schedule data type allows many different expressions. For example: "Every 8 hours"; "Three times a day"; "1/2 an hour before breakfast for 10 days from 23-Dec 2011:"; "15 Oct 2013, 17 Oct 2013 and 1 Nov 2013".  Sometimes, a rate can imply duration when expressed as total volume / duration (e.g.  500mL/2 hours implies a duration of 2 hours).  However, when rate doesn't imply duration (e.g. 250mL/hour), then the timing.repeat.duration is needed to convey the infuse over time period.</t>
@@ -1894,7 +1885,7 @@
     <t>Dosage.timing</t>
   </si>
   <si>
-    <t>QSET&lt;TS&gt; (GTS)</t>
+    <t>.effectiveTime</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.asNeeded[x]</t>
@@ -2094,29 +2085,16 @@
 </t>
   </si>
   <si>
-    <t>A fixed quantity (no comparator)</t>
-  </si>
-  <si>
-    <t>The comparator is not used on a SimpleQuantity</t>
-  </si>
-  <si>
-    <t>The context of use may frequently define what kind of quantity this is and therefore what kind of units can be used. The context of use may also restrict the values for the comparator.</t>
+    <t>Amount of medication per dose</t>
+  </si>
+  <si>
+    <t>Amount of medication per dose.</t>
   </si>
   <si>
     <t>GstdTabel902</t>
   </si>
   <si>
     <t>http://decor.nictiz.nl/fhir/ValueSet/2.16.840.1.113883.2.4.3.11.60.20.77.11.27--20160830202453</t>
-  </si>
-  <si>
-    <t>ele-1:All FHIR elements must have a @value or children {hasValue() | (children().count() &gt; id.count())}
-qty-3:If a code for the unit is present, the system SHALL also be present {code.empty() or system.exists()}sqty-1:The comparator is not used on a SimpleQuantity {comparator.empty()}</t>
-  </si>
-  <si>
-    <t>PQ, IVL&lt;PQ&gt;, MO, CO, depending on the values</t>
-  </si>
-  <si>
-    <t>SN (see also Range) or CQ</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.dose[x]:doseRange</t>
@@ -2127,12 +2105,6 @@
   <si>
     <t xml:space="preserve">Range
 </t>
-  </si>
-  <si>
-    <t>Amount of medication per dose</t>
-  </si>
-  <si>
-    <t>Amount of medication per dose.</t>
   </si>
   <si>
     <t>MedicationRequest.dosageInstruction.dose[x]:doseRange.id</t>
@@ -2343,6 +2315,10 @@
   </si>
   <si>
     <t>Indicates the specific details for the dispense or medication supply part of a medication request (also known as a Medication Prescription or Medication Order).  Note that this information is not always sent with the order.  There may be in some settings (e.g. hospitals) institutional or system support for completing the dispense details in the pharmacy department.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() | (children().count() &gt; id.count())}
+</t>
   </si>
   <si>
     <t>Message/Body/NewRx/MedicationPrescribed/ExpirationDate</t>
@@ -13263,7 +13239,7 @@
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
-        <v>547</v>
+        <v>85</v>
       </c>
       <c r="E81" s="2"/>
       <c r="F81" t="s" s="2">
@@ -13282,16 +13258,16 @@
         <v>85</v>
       </c>
       <c r="K81" t="s" s="2">
+        <v>547</v>
+      </c>
+      <c r="L81" t="s" s="2">
         <v>548</v>
       </c>
-      <c r="L81" t="s" s="2">
+      <c r="M81" t="s" s="2">
         <v>549</v>
       </c>
-      <c r="M81" t="s" s="2">
+      <c r="N81" t="s" s="2">
         <v>550</v>
-      </c>
-      <c r="N81" t="s" s="2">
-        <v>551</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" t="s" s="2">
@@ -13350,31 +13326,31 @@
         <v>84</v>
       </c>
       <c r="AI81" t="s" s="2">
-        <v>153</v>
+        <v>85</v>
       </c>
       <c r="AJ81" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AK81" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="AL81" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AM81" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="AK81" t="s" s="2">
+      <c r="AN81" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AO81" t="s" s="2">
         <v>553</v>
       </c>
-      <c r="AL81" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AM81" t="s" s="2">
+      <c r="AP81" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AQ81" t="s" s="2">
         <v>554</v>
-      </c>
-      <c r="AN81" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AO81" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AP81" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AQ81" t="s" s="2">
-        <v>555</v>
       </c>
       <c r="AR81" t="s" s="2">
         <v>85</v>
@@ -13385,10 +13361,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13512,10 +13488,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13641,14 +13617,14 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="E84" s="2"/>
       <c r="F84" t="s" s="2">
@@ -13667,17 +13643,17 @@
         <v>96</v>
       </c>
       <c r="K84" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="L84" t="s" s="2">
         <v>560</v>
       </c>
-      <c r="L84" t="s" s="2">
+      <c r="M84" t="s" s="2">
         <v>561</v>
-      </c>
-      <c r="M84" t="s" s="2">
-        <v>562</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="P84" t="s" s="2">
         <v>85</v>
@@ -13726,7 +13702,7 @@
         <v>85</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>83</v>
@@ -13759,7 +13735,7 @@
         <v>85</v>
       </c>
       <c r="AQ84" t="s" s="2">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AR84" t="s" s="2">
         <v>85</v>
@@ -13770,14 +13746,14 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" t="s" s="2">
@@ -13802,11 +13778,11 @@
         <v>21</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="N85" s="2"/>
       <c r="O85" t="s" s="2">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="P85" t="s" s="2">
         <v>85</v>
@@ -13855,7 +13831,7 @@
         <v>85</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>83</v>
@@ -13888,7 +13864,7 @@
         <v>85</v>
       </c>
       <c r="AQ85" t="s" s="2">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AR85" t="s" s="2">
         <v>85</v>
@@ -13899,14 +13875,14 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E86" s="2"/>
       <c r="F86" t="s" s="2">
@@ -13928,14 +13904,14 @@
         <v>194</v>
       </c>
       <c r="L86" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="M86" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="M86" t="s" s="2">
-        <v>574</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>85</v>
@@ -13964,25 +13940,25 @@
       </c>
       <c r="Y86" s="2"/>
       <c r="Z86" t="s" s="2">
+        <v>575</v>
+      </c>
+      <c r="AA86" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AB86" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AC86" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AD86" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AE86" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AF86" t="s" s="2">
         <v>576</v>
-      </c>
-      <c r="AA86" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AB86" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AC86" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AD86" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AE86" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AF86" t="s" s="2">
-        <v>577</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>83</v>
@@ -14015,7 +13991,7 @@
         <v>85</v>
       </c>
       <c r="AQ86" t="s" s="2">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AR86" t="s" s="2">
         <v>85</v>
@@ -14026,10 +14002,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -14055,10 +14031,10 @@
         <v>172</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>578</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>579</v>
-      </c>
-      <c r="M87" t="s" s="2">
-        <v>580</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -14109,7 +14085,7 @@
         <v>85</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>83</v>
@@ -14142,7 +14118,7 @@
         <v>85</v>
       </c>
       <c r="AQ87" t="s" s="2">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AR87" t="s" s="2">
         <v>85</v>
@@ -14153,14 +14129,14 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
-        <v>583</v>
+        <v>85</v>
       </c>
       <c r="E88" s="2"/>
       <c r="F88" t="s" s="2">
@@ -14176,22 +14152,22 @@
         <v>85</v>
       </c>
       <c r="J88" t="s" s="2">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="K88" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="L88" t="s" s="2">
+        <v>583</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>584</v>
       </c>
-      <c r="L88" t="s" s="2">
+      <c r="N88" t="s" s="2">
         <v>585</v>
       </c>
-      <c r="M88" t="s" s="2">
+      <c r="O88" t="s" s="2">
         <v>586</v>
-      </c>
-      <c r="N88" t="s" s="2">
-        <v>587</v>
-      </c>
-      <c r="O88" t="s" s="2">
-        <v>588</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>85</v>
@@ -14240,7 +14216,7 @@
         <v>85</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>83</v>
@@ -14249,10 +14225,10 @@
         <v>95</v>
       </c>
       <c r="AI88" t="s" s="2">
-        <v>153</v>
+        <v>85</v>
       </c>
       <c r="AJ88" t="s" s="2">
-        <v>552</v>
+        <v>85</v>
       </c>
       <c r="AK88" t="s" s="2">
         <v>85</v>
@@ -14273,21 +14249,21 @@
         <v>85</v>
       </c>
       <c r="AQ88" t="s" s="2">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AR88" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS88" t="s" s="2">
-        <v>138</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14313,13 +14289,13 @@
         <v>194</v>
       </c>
       <c r="L89" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="M89" t="s" s="2">
+        <v>591</v>
+      </c>
+      <c r="N89" t="s" s="2">
         <v>592</v>
-      </c>
-      <c r="M89" t="s" s="2">
-        <v>593</v>
-      </c>
-      <c r="N89" t="s" s="2">
-        <v>594</v>
       </c>
       <c r="O89" s="2"/>
       <c r="P89" t="s" s="2">
@@ -14345,13 +14321,13 @@
         <v>85</v>
       </c>
       <c r="X89" t="s" s="2">
+        <v>593</v>
+      </c>
+      <c r="Y89" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="Z89" t="s" s="2">
         <v>595</v>
-      </c>
-      <c r="Y89" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="Z89" t="s" s="2">
-        <v>597</v>
       </c>
       <c r="AA89" t="s" s="2">
         <v>85</v>
@@ -14367,7 +14343,7 @@
         <v>198</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>83</v>
@@ -14400,7 +14376,7 @@
         <v>85</v>
       </c>
       <c r="AQ89" t="s" s="2">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="AR89" t="s" s="2">
         <v>85</v>
@@ -14411,16 +14387,16 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
+        <v>598</v>
+      </c>
+      <c r="B90" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="C90" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="D90" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="B90" t="s" s="2">
-        <v>591</v>
-      </c>
-      <c r="C90" t="s" s="2">
-        <v>601</v>
-      </c>
-      <c r="D90" t="s" s="2">
-        <v>602</v>
       </c>
       <c r="E90" s="2"/>
       <c r="F90" t="s" s="2">
@@ -14442,13 +14418,13 @@
         <v>194</v>
       </c>
       <c r="L90" t="s" s="2">
+        <v>601</v>
+      </c>
+      <c r="M90" t="s" s="2">
+        <v>602</v>
+      </c>
+      <c r="N90" t="s" s="2">
         <v>603</v>
-      </c>
-      <c r="M90" t="s" s="2">
-        <v>604</v>
-      </c>
-      <c r="N90" t="s" s="2">
-        <v>605</v>
       </c>
       <c r="O90" s="2"/>
       <c r="P90" t="s" s="2">
@@ -14477,10 +14453,10 @@
         <v>118</v>
       </c>
       <c r="Y90" t="s" s="2">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="Z90" t="s" s="2">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>85</v>
@@ -14498,7 +14474,7 @@
         <v>85</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>83</v>
@@ -14531,7 +14507,7 @@
         <v>85</v>
       </c>
       <c r="AQ90" t="s" s="2">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="AR90" t="s" s="2">
         <v>85</v>
@@ -14542,10 +14518,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14571,16 +14547,16 @@
         <v>194</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="M91" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="N91" t="s" s="2">
         <v>609</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="O91" t="s" s="2">
         <v>610</v>
-      </c>
-      <c r="N91" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="O91" t="s" s="2">
-        <v>612</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>85</v>
@@ -14605,31 +14581,31 @@
         <v>85</v>
       </c>
       <c r="X91" t="s" s="2">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="Y91" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="Z91" t="s" s="2">
+        <v>612</v>
+      </c>
+      <c r="AA91" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AB91" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AC91" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AD91" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AE91" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AF91" t="s" s="2">
         <v>613</v>
-      </c>
-      <c r="Z91" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="AA91" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AB91" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AC91" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AD91" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AE91" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AF91" t="s" s="2">
-        <v>615</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>83</v>
@@ -14662,7 +14638,7 @@
         <v>85</v>
       </c>
       <c r="AQ91" t="s" s="2">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="AR91" t="s" s="2">
         <v>85</v>
@@ -14673,14 +14649,14 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E92" s="2"/>
       <c r="F92" t="s" s="2">
@@ -14702,14 +14678,14 @@
         <v>194</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="N92" s="2"/>
       <c r="O92" t="s" s="2">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="P92" t="s" s="2">
         <v>85</v>
@@ -14722,7 +14698,7 @@
         <v>85</v>
       </c>
       <c r="T92" t="s" s="2">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="U92" t="s" s="2">
         <v>85</v>
@@ -14737,28 +14713,28 @@
         <v>118</v>
       </c>
       <c r="Y92" t="s" s="2">
+        <v>621</v>
+      </c>
+      <c r="Z92" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="AA92" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AB92" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AC92" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AD92" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AE92" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AF92" t="s" s="2">
         <v>623</v>
-      </c>
-      <c r="Z92" t="s" s="2">
-        <v>624</v>
-      </c>
-      <c r="AA92" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AB92" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AC92" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AD92" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AE92" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AF92" t="s" s="2">
-        <v>625</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>83</v>
@@ -14791,7 +14767,7 @@
         <v>85</v>
       </c>
       <c r="AQ92" t="s" s="2">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="AR92" t="s" s="2">
         <v>85</v>
@@ -14802,10 +14778,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14929,10 +14905,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -15058,10 +15034,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -15189,10 +15165,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15320,10 +15296,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15349,16 +15325,16 @@
         <v>194</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>630</v>
+      </c>
+      <c r="M97" t="s" s="2">
+        <v>631</v>
+      </c>
+      <c r="N97" t="s" s="2">
         <v>632</v>
       </c>
-      <c r="M97" t="s" s="2">
+      <c r="O97" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="N97" t="s" s="2">
-        <v>634</v>
-      </c>
-      <c r="O97" t="s" s="2">
-        <v>635</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>85</v>
@@ -15383,31 +15359,31 @@
         <v>85</v>
       </c>
       <c r="X97" t="s" s="2">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="Y97" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="Z97" t="s" s="2">
+        <v>635</v>
+      </c>
+      <c r="AA97" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AB97" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AC97" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AD97" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AE97" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AF97" t="s" s="2">
         <v>636</v>
-      </c>
-      <c r="Z97" t="s" s="2">
-        <v>637</v>
-      </c>
-      <c r="AA97" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AB97" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AC97" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AD97" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AE97" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AF97" t="s" s="2">
-        <v>638</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15440,7 +15416,7 @@
         <v>85</v>
       </c>
       <c r="AQ97" t="s" s="2">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="AR97" t="s" s="2">
         <v>85</v>
@@ -15451,14 +15427,14 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="E98" s="2"/>
       <c r="F98" t="s" s="2">
@@ -15477,19 +15453,19 @@
         <v>96</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="L98" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="M98" t="s" s="2">
         <v>642</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>643</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="O98" t="s" s="2">
         <v>644</v>
-      </c>
-      <c r="N98" t="s" s="2">
-        <v>645</v>
-      </c>
-      <c r="O98" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>85</v>
@@ -15536,7 +15512,7 @@
         <v>198</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15569,7 +15545,7 @@
         <v>85</v>
       </c>
       <c r="AQ98" t="s" s="2">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="AR98" t="s" s="2">
         <v>85</v>
@@ -15580,13 +15556,13 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C99" t="s" s="2">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D99" t="s" s="2">
         <v>85</v>
@@ -15605,22 +15581,22 @@
         <v>85</v>
       </c>
       <c r="J99" t="s" s="2">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="K99" t="s" s="2">
+        <v>648</v>
+      </c>
+      <c r="L99" t="s" s="2">
+        <v>649</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>650</v>
       </c>
-      <c r="L99" t="s" s="2">
-        <v>651</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>652</v>
-      </c>
       <c r="N99" t="s" s="2">
-        <v>653</v>
+        <v>643</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>85</v>
@@ -15648,10 +15624,10 @@
         <v>238</v>
       </c>
       <c r="Y99" t="s" s="2">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="Z99" t="s" s="2">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="AA99" t="s" s="2">
         <v>85</v>
@@ -15669,7 +15645,7 @@
         <v>85</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15678,10 +15654,10 @@
         <v>95</v>
       </c>
       <c r="AI99" t="s" s="2">
-        <v>153</v>
+        <v>85</v>
       </c>
       <c r="AJ99" t="s" s="2">
-        <v>656</v>
+        <v>85</v>
       </c>
       <c r="AK99" t="s" s="2">
         <v>85</v>
@@ -15702,24 +15678,24 @@
         <v>85</v>
       </c>
       <c r="AQ99" t="s" s="2">
-        <v>657</v>
+        <v>637</v>
       </c>
       <c r="AR99" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS99" t="s" s="2">
-        <v>658</v>
+        <v>85</v>
       </c>
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>659</v>
+        <v>653</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C100" t="s" s="2">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="D100" t="s" s="2">
         <v>85</v>
@@ -15741,19 +15717,19 @@
         <v>96</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>663</v>
+        <v>650</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="O100" t="s" s="2">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>85</v>
@@ -15802,7 +15778,7 @@
         <v>85</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15835,7 +15811,7 @@
         <v>85</v>
       </c>
       <c r="AQ100" t="s" s="2">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="AR100" t="s" s="2">
         <v>85</v>
@@ -15846,10 +15822,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>664</v>
+        <v>656</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>665</v>
+        <v>657</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15973,10 +15949,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>666</v>
+        <v>658</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>667</v>
+        <v>659</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -16102,10 +16078,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>668</v>
+        <v>660</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>669</v>
+        <v>661</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -16128,16 +16104,16 @@
         <v>96</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>670</v>
+        <v>662</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>671</v>
+        <v>663</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -16166,10 +16142,10 @@
         <v>238</v>
       </c>
       <c r="Y103" t="s" s="2">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="Z103" t="s" s="2">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>85</v>
@@ -16187,7 +16163,7 @@
         <v>85</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>83</v>
@@ -16196,7 +16172,7 @@
         <v>95</v>
       </c>
       <c r="AI103" t="s" s="2">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="AJ103" t="s" s="2">
         <v>85</v>
@@ -16220,21 +16196,21 @@
         <v>85</v>
       </c>
       <c r="AQ103" t="s" s="2">
-        <v>675</v>
+        <v>667</v>
       </c>
       <c r="AR103" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS103" t="s" s="2">
-        <v>676</v>
+        <v>668</v>
       </c>
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>677</v>
+        <v>669</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>678</v>
+        <v>670</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -16257,16 +16233,16 @@
         <v>96</v>
       </c>
       <c r="K104" t="s" s="2">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>680</v>
+        <v>672</v>
       </c>
       <c r="N104" t="s" s="2">
-        <v>681</v>
+        <v>673</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -16295,10 +16271,10 @@
         <v>238</v>
       </c>
       <c r="Y104" t="s" s="2">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="Z104" t="s" s="2">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="AA104" t="s" s="2">
         <v>85</v>
@@ -16316,7 +16292,7 @@
         <v>85</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>682</v>
+        <v>674</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>83</v>
@@ -16325,7 +16301,7 @@
         <v>95</v>
       </c>
       <c r="AI104" t="s" s="2">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="AJ104" t="s" s="2">
         <v>85</v>
@@ -16349,25 +16325,25 @@
         <v>85</v>
       </c>
       <c r="AQ104" t="s" s="2">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="AR104" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS104" t="s" s="2">
-        <v>684</v>
+        <v>676</v>
       </c>
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="E105" s="2"/>
       <c r="F105" t="s" s="2">
@@ -16386,19 +16362,19 @@
         <v>96</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>688</v>
+        <v>680</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="N105" t="s" s="2">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="O105" t="s" s="2">
-        <v>691</v>
+        <v>683</v>
       </c>
       <c r="P105" t="s" s="2">
         <v>85</v>
@@ -16447,7 +16423,7 @@
         <v>85</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>692</v>
+        <v>684</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>83</v>
@@ -16480,7 +16456,7 @@
         <v>85</v>
       </c>
       <c r="AQ105" t="s" s="2">
-        <v>693</v>
+        <v>685</v>
       </c>
       <c r="AR105" t="s" s="2">
         <v>85</v>
@@ -16491,10 +16467,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -16618,10 +16594,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -16747,10 +16723,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -16773,13 +16749,13 @@
         <v>96</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>698</v>
+        <v>690</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -16809,10 +16785,10 @@
         <v>238</v>
       </c>
       <c r="Y108" t="s" s="2">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="Z108" t="s" s="2">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="AA108" t="s" s="2">
         <v>85</v>
@@ -16830,7 +16806,7 @@
         <v>85</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>83</v>
@@ -16863,7 +16839,7 @@
         <v>85</v>
       </c>
       <c r="AQ108" t="s" s="2">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="AR108" t="s" s="2">
         <v>85</v>
@@ -16874,10 +16850,10 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -16900,13 +16876,13 @@
         <v>96</v>
       </c>
       <c r="K109" t="s" s="2">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="N109" s="2"/>
       <c r="O109" s="2"/>
@@ -16957,7 +16933,7 @@
         <v>85</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>83</v>
@@ -16990,7 +16966,7 @@
         <v>85</v>
       </c>
       <c r="AQ109" t="s" s="2">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="AR109" t="s" s="2">
         <v>85</v>
@@ -17001,10 +16977,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -17027,19 +17003,19 @@
         <v>96</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="N110" t="s" s="2">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="O110" t="s" s="2">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="P110" t="s" s="2">
         <v>85</v>
@@ -17088,7 +17064,7 @@
         <v>85</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>712</v>
+        <v>704</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>83</v>
@@ -17121,7 +17097,7 @@
         <v>85</v>
       </c>
       <c r="AQ110" t="s" s="2">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="AR110" t="s" s="2">
         <v>85</v>
@@ -17132,10 +17108,10 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>714</v>
+        <v>706</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>714</v>
+        <v>706</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -17158,17 +17134,17 @@
         <v>96</v>
       </c>
       <c r="K111" t="s" s="2">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>715</v>
+        <v>707</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>716</v>
+        <v>708</v>
       </c>
       <c r="N111" s="2"/>
       <c r="O111" t="s" s="2">
-        <v>717</v>
+        <v>709</v>
       </c>
       <c r="P111" t="s" s="2">
         <v>85</v>
@@ -17217,7 +17193,7 @@
         <v>85</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>83</v>
@@ -17250,7 +17226,7 @@
         <v>85</v>
       </c>
       <c r="AQ111" t="s" s="2">
-        <v>713</v>
+        <v>705</v>
       </c>
       <c r="AR111" t="s" s="2">
         <v>85</v>
@@ -17261,14 +17237,14 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
-        <v>720</v>
+        <v>712</v>
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
@@ -17287,19 +17263,19 @@
         <v>96</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>721</v>
+        <v>713</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>722</v>
+        <v>714</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="N112" t="s" s="2">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="O112" t="s" s="2">
-        <v>725</v>
+        <v>717</v>
       </c>
       <c r="P112" t="s" s="2">
         <v>85</v>
@@ -17348,7 +17324,7 @@
         <v>85</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>726</v>
+        <v>718</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>83</v>
@@ -17381,7 +17357,7 @@
         <v>85</v>
       </c>
       <c r="AQ112" t="s" s="2">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="AR112" t="s" s="2">
         <v>85</v>
@@ -17392,10 +17368,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -17421,10 +17397,10 @@
         <v>462</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -17475,7 +17451,7 @@
         <v>85</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>83</v>
@@ -17487,7 +17463,7 @@
         <v>85</v>
       </c>
       <c r="AJ113" t="s" s="2">
-        <v>552</v>
+        <v>723</v>
       </c>
       <c r="AK113" t="s" s="2">
         <v>85</v>
@@ -17505,10 +17481,10 @@
         <v>85</v>
       </c>
       <c r="AP113" t="s" s="2">
-        <v>731</v>
+        <v>724</v>
       </c>
       <c r="AQ113" t="s" s="2">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="AR113" t="s" s="2">
         <v>85</v>
@@ -17519,10 +17495,10 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -17646,10 +17622,10 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -17775,10 +17751,10 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -17904,10 +17880,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -17930,19 +17906,19 @@
         <v>85</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>737</v>
+        <v>730</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>739</v>
+        <v>732</v>
       </c>
       <c r="N117" t="s" s="2">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="O117" t="s" s="2">
-        <v>741</v>
+        <v>734</v>
       </c>
       <c r="P117" t="s" s="2">
         <v>85</v>
@@ -17991,7 +17967,7 @@
         <v>85</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>83</v>
@@ -18021,10 +17997,10 @@
         <v>85</v>
       </c>
       <c r="AP117" t="s" s="2">
-        <v>742</v>
+        <v>735</v>
       </c>
       <c r="AQ117" t="s" s="2">
-        <v>743</v>
+        <v>736</v>
       </c>
       <c r="AR117" t="s" s="2">
         <v>85</v>
@@ -18035,10 +18011,10 @@
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -18061,16 +18037,16 @@
         <v>85</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>745</v>
+        <v>738</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>747</v>
+        <v>740</v>
       </c>
       <c r="N118" t="s" s="2">
-        <v>748</v>
+        <v>741</v>
       </c>
       <c r="O118" s="2"/>
       <c r="P118" t="s" s="2">
@@ -18120,7 +18096,7 @@
         <v>85</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>83</v>
@@ -18150,24 +18126,24 @@
         <v>85</v>
       </c>
       <c r="AP118" t="s" s="2">
-        <v>749</v>
+        <v>742</v>
       </c>
       <c r="AQ118" t="s" s="2">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="AR118" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS118" t="s" s="2">
-        <v>751</v>
+        <v>744</v>
       </c>
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -18190,13 +18166,13 @@
         <v>85</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>754</v>
+        <v>747</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
@@ -18247,7 +18223,7 @@
         <v>85</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>83</v>
@@ -18277,24 +18253,24 @@
         <v>85</v>
       </c>
       <c r="AP119" t="s" s="2">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="AQ119" t="s" s="2">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="AR119" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS119" t="s" s="2">
-        <v>757</v>
+        <v>750</v>
       </c>
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -18317,16 +18293,16 @@
         <v>85</v>
       </c>
       <c r="K120" t="s" s="2">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="N120" t="s" s="2">
-        <v>762</v>
+        <v>755</v>
       </c>
       <c r="O120" s="2"/>
       <c r="P120" t="s" s="2">
@@ -18376,7 +18352,7 @@
         <v>85</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>83</v>
@@ -18406,10 +18382,10 @@
         <v>85</v>
       </c>
       <c r="AP120" t="s" s="2">
-        <v>763</v>
+        <v>756</v>
       </c>
       <c r="AQ120" t="s" s="2">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="AR120" t="s" s="2">
         <v>85</v>
@@ -18420,10 +18396,10 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -18446,13 +18422,13 @@
         <v>85</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="L121" t="s" s="2">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>768</v>
+        <v>761</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -18503,7 +18479,7 @@
         <v>85</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>83</v>
@@ -18536,7 +18512,7 @@
         <v>85</v>
       </c>
       <c r="AQ121" t="s" s="2">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="AR121" t="s" s="2">
         <v>508</v>
@@ -18547,10 +18523,10 @@
     </row>
     <row r="122" hidden="true">
       <c r="A122" t="s" s="2">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -18576,10 +18552,10 @@
         <v>462</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
@@ -18630,7 +18606,7 @@
         <v>85</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>83</v>
@@ -18642,7 +18618,7 @@
         <v>85</v>
       </c>
       <c r="AJ122" t="s" s="2">
-        <v>552</v>
+        <v>723</v>
       </c>
       <c r="AK122" t="s" s="2">
         <v>85</v>
@@ -18660,10 +18636,10 @@
         <v>85</v>
       </c>
       <c r="AP122" t="s" s="2">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="AQ122" t="s" s="2">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="AR122" t="s" s="2">
         <v>85</v>
@@ -18674,10 +18650,10 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -18801,10 +18777,10 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -18930,10 +18906,10 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>777</v>
+        <v>770</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -19059,10 +19035,10 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>778</v>
+        <v>771</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>778</v>
+        <v>771</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -19088,13 +19064,13 @@
         <v>360</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>779</v>
+        <v>772</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>780</v>
+        <v>773</v>
       </c>
       <c r="N126" t="s" s="2">
-        <v>781</v>
+        <v>774</v>
       </c>
       <c r="O126" s="2"/>
       <c r="P126" t="s" s="2">
@@ -19144,7 +19120,7 @@
         <v>85</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>778</v>
+        <v>771</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>95</v>
@@ -19174,24 +19150,24 @@
         <v>85</v>
       </c>
       <c r="AP126" t="s" s="2">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="AQ126" t="s" s="2">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="AR126" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS126" t="s" s="2">
-        <v>783</v>
+        <v>776</v>
       </c>
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>784</v>
+        <v>777</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>784</v>
+        <v>777</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -19217,10 +19193,10 @@
         <v>194</v>
       </c>
       <c r="L127" t="s" s="2">
-        <v>785</v>
+        <v>778</v>
       </c>
       <c r="M127" t="s" s="2">
-        <v>786</v>
+        <v>779</v>
       </c>
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
@@ -19247,13 +19223,13 @@
         <v>85</v>
       </c>
       <c r="X127" t="s" s="2">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="Y127" t="s" s="2">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="Z127" t="s" s="2">
-        <v>788</v>
+        <v>781</v>
       </c>
       <c r="AA127" t="s" s="2">
         <v>85</v>
@@ -19271,7 +19247,7 @@
         <v>85</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>784</v>
+        <v>777</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>83</v>
@@ -19301,24 +19277,24 @@
         <v>85</v>
       </c>
       <c r="AP127" t="s" s="2">
-        <v>789</v>
+        <v>782</v>
       </c>
       <c r="AQ127" t="s" s="2">
-        <v>790</v>
+        <v>783</v>
       </c>
       <c r="AR127" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AS127" t="s" s="2">
-        <v>791</v>
+        <v>784</v>
       </c>
     </row>
     <row r="128" hidden="true">
       <c r="A128" t="s" s="2">
-        <v>792</v>
+        <v>785</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>792</v>
+        <v>785</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -19341,13 +19317,13 @@
         <v>85</v>
       </c>
       <c r="K128" t="s" s="2">
-        <v>793</v>
+        <v>786</v>
       </c>
       <c r="L128" t="s" s="2">
-        <v>794</v>
+        <v>787</v>
       </c>
       <c r="M128" t="s" s="2">
-        <v>795</v>
+        <v>788</v>
       </c>
       <c r="N128" s="2"/>
       <c r="O128" s="2"/>
@@ -19398,7 +19374,7 @@
         <v>85</v>
       </c>
       <c r="AF128" t="s" s="2">
-        <v>792</v>
+        <v>785</v>
       </c>
       <c r="AG128" t="s" s="2">
         <v>83</v>
@@ -19425,13 +19401,13 @@
         <v>85</v>
       </c>
       <c r="AO128" t="s" s="2">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="AP128" t="s" s="2">
-        <v>789</v>
+        <v>782</v>
       </c>
       <c r="AQ128" t="s" s="2">
-        <v>797</v>
+        <v>790</v>
       </c>
       <c r="AR128" t="s" s="2">
         <v>85</v>
@@ -19442,14 +19418,14 @@
     </row>
     <row r="129" hidden="true">
       <c r="A129" t="s" s="2">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
-        <v>799</v>
+        <v>792</v>
       </c>
       <c r="E129" s="2"/>
       <c r="F129" t="s" s="2">
@@ -19468,13 +19444,13 @@
         <v>85</v>
       </c>
       <c r="K129" t="s" s="2">
-        <v>800</v>
+        <v>793</v>
       </c>
       <c r="L129" t="s" s="2">
-        <v>801</v>
+        <v>794</v>
       </c>
       <c r="M129" t="s" s="2">
-        <v>802</v>
+        <v>795</v>
       </c>
       <c r="N129" s="2"/>
       <c r="O129" s="2"/>
@@ -19525,7 +19501,7 @@
         <v>85</v>
       </c>
       <c r="AF129" t="s" s="2">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="AG129" t="s" s="2">
         <v>83</v>
@@ -19558,7 +19534,7 @@
         <v>85</v>
       </c>
       <c r="AQ129" t="s" s="2">
-        <v>803</v>
+        <v>796</v>
       </c>
       <c r="AR129" t="s" s="2">
         <v>85</v>
@@ -19569,10 +19545,10 @@
     </row>
     <row r="130" hidden="true">
       <c r="A130" t="s" s="2">
-        <v>804</v>
+        <v>797</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>804</v>
+        <v>797</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -19595,16 +19571,16 @@
         <v>85</v>
       </c>
       <c r="K130" t="s" s="2">
-        <v>805</v>
+        <v>798</v>
       </c>
       <c r="L130" t="s" s="2">
-        <v>806</v>
+        <v>799</v>
       </c>
       <c r="M130" t="s" s="2">
-        <v>807</v>
+        <v>800</v>
       </c>
       <c r="N130" t="s" s="2">
-        <v>808</v>
+        <v>801</v>
       </c>
       <c r="O130" s="2"/>
       <c r="P130" t="s" s="2">
@@ -19654,7 +19630,7 @@
         <v>85</v>
       </c>
       <c r="AF130" t="s" s="2">
-        <v>804</v>
+        <v>797</v>
       </c>
       <c r="AG130" t="s" s="2">
         <v>83</v>
@@ -19681,13 +19657,13 @@
         <v>85</v>
       </c>
       <c r="AO130" t="s" s="2">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="AP130" t="s" s="2">
         <v>85</v>
       </c>
       <c r="AQ130" t="s" s="2">
-        <v>810</v>
+        <v>803</v>
       </c>
       <c r="AR130" t="s" s="2">
         <v>85</v>

</xml_diff>